<commit_message>
Add Tesseract OCR dependency and configuration for image document parsing
</commit_message>
<xml_diff>
--- a/src/main/resources/test-files/report.xlsx
+++ b/src/main/resources/test-files/report.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Даниил\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Даниил\Desktop\apache-poi-elasticsearch-orestration-minikube\apache-poi-elasticsearch-orestration-minikube\src\main\resources\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Дата</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t>Сидоров В.Г</t>
+  </si>
+  <si>
+    <t>Брянск</t>
+  </si>
+  <si>
+    <t>Ноутбук Colorful</t>
+  </si>
+  <si>
+    <t>Андреев А.В</t>
   </si>
 </sst>
 </file>
@@ -408,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" customWidth="1"/>
@@ -536,6 +545,35 @@
         <v>17</v>
       </c>
     </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>44947</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>240000</v>
+      </c>
+      <c r="G5">
+        <v>720000</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update test Excel file with sales data for AI analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/test-files/report.xlsx
+++ b/src/main/resources/test-files/report.xlsx
@@ -26,79 +26,79 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
-    <t>Дата</t>
-  </si>
-  <si>
-    <t>Регион</t>
-  </si>
-  <si>
-    <t>Продукт</t>
-  </si>
-  <si>
-    <t>Количество</t>
-  </si>
-  <si>
-    <t>Цена</t>
-  </si>
-  <si>
-    <t>Сумма</t>
-  </si>
-  <si>
-    <t>Менеджер</t>
-  </si>
-  <si>
-    <t>Статус</t>
-  </si>
-  <si>
-    <t>Москва</t>
-  </si>
-  <si>
-    <t>Ноутбук Dell XPS</t>
-  </si>
-  <si>
-    <t>Электроника</t>
-  </si>
-  <si>
-    <t>Иванов А.А.</t>
-  </si>
-  <si>
-    <t>Выполнен</t>
-  </si>
-  <si>
-    <t>Монитор Samsung 27"</t>
-  </si>
-  <si>
-    <t>Петров Б.В.</t>
-  </si>
-  <si>
-    <t>Казань</t>
-  </si>
-  <si>
-    <t>Клавиатура Logitech</t>
-  </si>
-  <si>
-    <t>В обработке</t>
-  </si>
-  <si>
-    <t>Категории</t>
-  </si>
-  <si>
-    <t>Санкт_Петербург</t>
-  </si>
-  <si>
-    <t>Переферия</t>
-  </si>
-  <si>
-    <t>Сидоров В.Г</t>
-  </si>
-  <si>
-    <t>Брянск</t>
-  </si>
-  <si>
-    <t>Ноутбук Colorful</t>
-  </si>
-  <si>
-    <t>Андреев А.В</t>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Counts</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Moscow</t>
+  </si>
+  <si>
+    <t>St. Petersburg</t>
+  </si>
+  <si>
+    <t>Kazan</t>
+  </si>
+  <si>
+    <t>Bryansk</t>
+  </si>
+  <si>
+    <t>Dell XPS Laptop</t>
+  </si>
+  <si>
+    <t>Samsung 27" Monitor</t>
+  </si>
+  <si>
+    <t>Logitech Keyboard</t>
+  </si>
+  <si>
+    <t>Colorful Laptop</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Paraphernalia</t>
+  </si>
+  <si>
+    <t>Ivanov A.A.</t>
+  </si>
+  <si>
+    <t>Petrov B.V.</t>
+  </si>
+  <si>
+    <t>Sidorov V.G.</t>
+  </si>
+  <si>
+    <t>Andreev A.V.</t>
   </si>
 </sst>
 </file>
@@ -440,22 +440,22 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -463,13 +463,13 @@
         <v>44576</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -481,10 +481,10 @@
         <v>600000</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -492,13 +492,13 @@
         <v>44577</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
         <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -510,10 +510,10 @@
         <v>350000</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -521,10 +521,10 @@
         <v>44578</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
@@ -539,10 +539,10 @@
         <v>125000</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -550,13 +550,13 @@
         <v>44947</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -571,7 +571,7 @@
         <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>